<commit_message>
Update reports 2026-10-30 10:06
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-30.xlsx
+++ b/gex_pivot_levels_2026-10-30.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$37.11M</t>
+          <t>-$36.60M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$42.45M</t>
+          <t>+$41.93M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -573,12 +573,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$50.15M</t>
+          <t>-$56.03M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$53.80M</t>
+          <t>+$59.58M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -606,12 +606,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$6.50M</t>
+          <t>-$9.13M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$8.63M</t>
+          <t>+$11.28M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -639,12 +639,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>-$45.56M</t>
+          <t>-$40.82M</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>+$55.12M</t>
+          <t>+$49.37M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$7.51M</t>
+          <t>-$6.79M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$8.83M</t>
+          <t>+$7.98M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -705,12 +705,12 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-$20.07M</t>
+          <t>-$19.45M</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>+$34.61M</t>
+          <t>+$33.55M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>-$83.11M</t>
+          <t>-$101.04M</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>+$120.70M</t>
+          <t>+$138.64M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -758,387 +758,420 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="2" t="n">
+        <v>7594.86</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>7635</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>-$3.19M</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>+$27.72M</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
         <v>7599.86</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B10" s="2" t="n">
         <v>7640</v>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>-$3.19M</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>+$28.02M</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>-$3.23M</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>+$28.41M</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>7609.86</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7650</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>-$63.92M</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>+$104.34M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>7609.86</v>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>7650</v>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>-$60.60M</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>+$98.92M</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>7614.86</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>7655</v>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>-$5.60M</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>+$12.22M</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
+        <v>7614.86</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>7655</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>-$5.98M</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>+$13.06M</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
         <v>7626.46</v>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B13" s="2" t="n">
         <v>764</v>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>+$10.65M</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>+$50.50M</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>+$3.27M</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>+$61.86M</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="n">
-        <v>7629.86</v>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>7670</v>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>-$20.72M</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>+$28.82M</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
+        <v>7629.86</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>7670</v>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>-$22.82M</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>+$31.74M</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
         <v>7636.5</v>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B15" s="5" t="n">
         <v>765</v>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>-$262.47M</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>+$321.87M</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>-$253.69M</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>+$320.44M</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>7649.86</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>7690</v>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>-$11.24M</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>+$20.76M</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
+        <v>7649.86</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>7690</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>-$13.08M</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>+$24.16M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>7654.86</v>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>7695</v>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>-$984.35K</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>+$8.59M</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>-$1.14M</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>+$9.94M</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
+    <row r="18">
+      <c r="A18" s="5" t="n">
         <v>7659.86</v>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B18" s="5" t="n">
         <v>7700</v>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>-$22.78M</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>+$84.30M</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>-$26.17M</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>+$96.85M</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>7684.86</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>7725</v>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>+$2.83M</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>+$19.82M</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
+        <v>7684.86</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>7725</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>+$3.15M</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>+$22.02M</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
         <v>7686.67</v>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B20" s="5" t="n">
         <v>770</v>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>+$26.28M</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>+$162.02M</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>+$46.88M</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>+$164.84M</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>7709.86</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>-$794.43K</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>+$18.92M</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>7709.86</v>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>-$794.43K</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>+$18.92M</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G20"/>
+  <autoFilter ref="A1:G21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2926,7 +2959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3000,12 +3033,12 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>-$262.47M</t>
+          <t>-$253.69M</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>+$321.87M</t>
+          <t>+$320.44M</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -3020,38 +3053,42 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="5" t="n">
         <v>7686.67</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="5" t="n">
         <v>770</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>+$26.28M</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>+$162.02M</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>+$46.88M</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>+$164.84M</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -3072,12 +3109,12 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>-$83.11M</t>
+          <t>-$101.04M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>+$120.70M</t>
+          <t>+$138.64M</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -3148,12 +3185,12 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>-$60.60M</t>
+          <t>-$63.92M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>+$98.92M</t>
+          <t>+$104.34M</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -3170,28 +3207,28 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>28727.51</v>
+        <v>7659.86</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>710</v>
+        <v>7700</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>-$52.36M</t>
+          <t>-$26.17M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>+$92.04M</t>
+          <t>+$96.85M</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -3212,10 +3249,10 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>28316.48</v>
+        <v>28727.51</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -3224,12 +3261,12 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>-$82.52M</t>
+          <t>-$52.36M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>+$91.42M</t>
+          <t>+$92.04M</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -3246,28 +3283,28 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>7659.86</v>
+        <v>28316.48</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>7700</v>
+        <v>700</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>-$22.78M</t>
+          <t>-$82.52M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>+$84.30M</t>
+          <t>+$91.42M</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -3320,68 +3357,68 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>28522</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>705</v>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>-$30.54M</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>+$61.15M</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>7626.46</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>764</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>+$3.27M</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>+$61.86M</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>7559.86</v>
+        <v>28522</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>7600</v>
+        <v>705</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>-$45.56M</t>
+          <t>-$30.54M</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>+$55.12M</t>
+          <t>+$61.15M</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -3414,12 +3451,12 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>-$50.15M</t>
+          <t>-$56.03M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>+$53.80M</t>
+          <t>+$59.58M</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -3434,40 +3471,40 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
-        <v>7626.46</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>764</v>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>+$10.65M</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>+$50.50M</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="B14" s="5" t="n">
+        <v>7559.86</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>7600</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>-$40.82M</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>+$49.37M</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3600,12 +3637,12 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>-$37.11M</t>
+          <t>-$36.60M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>+$42.45M</t>
+          <t>+$41.93M</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -3634,12 +3671,12 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>-$20.07M</t>
+          <t>-$19.45M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>+$34.61M</t>
+          <t>+$33.55M</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -3656,28 +3693,28 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>4036.99</v>
+        <v>7629.86</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>82</v>
+        <v>7670</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>+$27.88M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>-$22.82M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>+$29.60M</t>
+          <t>+$31.74M</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -3687,217 +3724,217 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>4036.99</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>+$27.88M</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>+$29.60M</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
+      <c r="B22" s="5" t="n">
         <v>28110.97</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C22" s="5" t="n">
         <v>695</v>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>-$25.06M</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>+$29.40M</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B23" s="2" t="n">
         <v>2796.68</v>
       </c>
-      <c r="C22" s="2" t="n">
+      <c r="C23" s="2" t="n">
         <v>278</v>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>-$3.18M</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>+$29.30M</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
-        <v>7629.86</v>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>7670</v>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="B24" s="2" t="n">
+        <v>7599.86</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>7640</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>-$20.72M</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>+$28.82M</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>7599.86</v>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>7640</v>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>-$3.19M</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>+$28.02M</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>-$3.23M</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>+$28.41M</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>28809.72</v>
+        <v>7594.86</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>712</v>
+        <v>7635</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>-$16.54M</t>
+          <t>-$3.19M</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>+$26.95M</t>
+          <t>+$27.72M</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>2816.8</v>
+        <v>28809.72</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>280</v>
+        <v>712</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>+$4.85M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>-$16.54M</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>+$23.87M</t>
+          <t>+$26.95M</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -3926,12 +3963,12 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>-$11.24M</t>
+          <t>-$13.08M</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>+$20.76M</t>
+          <t>+$24.16M</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -3944,28 +3981,28 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>7684.86</v>
+        <v>2816.8</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>7725</v>
+        <v>280</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>+$2.83M</t>
+          <t>+$4.85M</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>+$19.82M</t>
+          <t>+$23.87M</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -3978,112 +4015,108 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>2877.16</v>
+        <v>7684.86</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>286</v>
+        <v>7725</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>+$17.83M</t>
+          <t>+$3.15M</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+$19.44M</t>
+          <t>+$22.02M</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>7709.86</v>
+        <v>2877.16</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>7750</v>
+        <v>286</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>-$794.43K</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>+$17.83M</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>+$18.92M</t>
+          <t>+$19.44M</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>28563.1</v>
+        <v>7709.86</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>706</v>
+        <v>7750</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>+$3.60M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>-$794.43K</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>+$18.34M</t>
+          <t>+$18.92M</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -4092,70 +4125,70 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
+        <v>28563.1</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>706</v>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>+$3.60M</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>+$18.34M</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
         <v>29344.05</v>
       </c>
-      <c r="C32" s="2" t="n">
+      <c r="C33" s="2" t="n">
         <v>725</v>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>-$1.38M</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>+$17.44M</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>4019.53</v>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>370</v>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>-$7.82M</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>+$16.29M</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -4164,108 +4197,108 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
+        <v>4019.53</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>-$7.82M</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>+$16.29M</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
         <v>3997.81</v>
       </c>
-      <c r="C34" s="5" t="n">
+      <c r="C35" s="5" t="n">
         <v>368</v>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>-$12.91M</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>+$14.24M</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B36" s="2" t="n">
         <v>7614.86</v>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C36" s="2" t="n">
         <v>7655</v>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>-$5.60M</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>+$12.22M</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>-$5.98M</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>+$13.06M</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>4086.22</v>
-      </c>
-      <c r="C36" s="5" t="n">
-        <v>83</v>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
-        <is>
-          <t>+$11.09M</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>+$11.94M</t>
-        </is>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4278,70 +4311,70 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
+        <v>4086.22</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>+$11.09M</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>+$11.94M</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
         <v>4184.68</v>
       </c>
-      <c r="C37" s="5" t="n">
+      <c r="C38" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>+$9.88M</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>+$11.32M</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n">
-        <v>7564.86</v>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>7605</v>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>-$7.51M</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>+$8.83M</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4366,12 +4399,12 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>-$6.50M</t>
+          <t>-$9.13M</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>+$8.63M</t>
+          <t>+$11.28M</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -4404,12 +4437,12 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>-$984.35K</t>
+          <t>-$1.14M</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>+$8.59M</t>
+          <t>+$9.94M</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -4426,28 +4459,28 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>28398.69</v>
+        <v>7564.86</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>702</v>
+        <v>7605</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>-$5.36M</t>
+          <t>-$6.79M</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>+$7.92M</t>
+          <t>+$7.98M</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -4468,10 +4501,10 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>28768.61</v>
+        <v>28398.69</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>711</v>
+        <v>702</v>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
@@ -4480,12 +4513,12 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>-$4.67M</t>
+          <t>-$5.36M</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>+$7.40M</t>
+          <t>+$7.92M</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -4502,146 +4535,150 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>28768.61</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>711</v>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>-$4.67M</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>+$7.40M</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B44" s="2" t="n">
         <v>4073.85</v>
       </c>
-      <c r="C43" s="2" t="n">
+      <c r="C44" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr">
+      <c r="E44" s="8" t="inlineStr">
         <is>
           <t>+$402.42K</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>+$6.85M</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="H44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B44" s="5" t="n">
+      <c r="B45" s="5" t="n">
         <v>103.67</v>
       </c>
-      <c r="C44" s="5" t="n">
+      <c r="C45" s="5" t="n">
         <v>169</v>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
+      <c r="E45" s="9" t="inlineStr">
         <is>
           <t>+$6.21M</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>+$6.66M</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="n">
-        <v>2892.25</v>
-      </c>
-      <c r="C45" s="2" t="n">
-        <v>287.5</v>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>+$5.38M</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>+$5.39M</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>4041.26</v>
+        <v>2892.25</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>372</v>
+        <v>287.5</v>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>+$2.37M</t>
+          <t>+$5.38M</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>+$5.30M</t>
+          <t>+$5.39M</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -4650,244 +4687,244 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>4008.67</v>
+        <v>4041.26</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>-$751.71K</t>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>+$2.37M</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>+$4.71M</t>
+          <t>+$5.30M</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>4008.67</v>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>369</v>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>-$751.71K</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>+$4.71M</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B48" s="2" t="n">
+      <c r="B49" s="2" t="n">
         <v>28234.28</v>
       </c>
-      <c r="C48" s="2" t="n">
+      <c r="C49" s="2" t="n">
         <v>698</v>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>-$2.78M</t>
         </is>
       </c>
-      <c r="F48" s="3" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>+$3.29M</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n">
+      <c r="B50" s="5" t="n">
         <v>4128.17</v>
       </c>
-      <c r="C49" s="5" t="n">
+      <c r="C50" s="5" t="n">
         <v>380</v>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E50" s="9" t="inlineStr">
         <is>
           <t>+$2.67M</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>+$3.13M</t>
         </is>
       </c>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H49" s="6" t="inlineStr">
+      <c r="H50" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>101.21</v>
-      </c>
-      <c r="C50" s="2" t="n">
-        <v>165</v>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>+$188.14K</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>+$2.94M</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>27946.56</v>
+        <v>101.21</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>691</v>
+        <v>165</v>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>-$2.37M</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>+$188.14K</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>+$2.82M</t>
+          <t>+$2.94M</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>3943.49</v>
+        <v>27946.56</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>363</v>
+        <v>691</v>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>-$2.49M</t>
+          <t>-$2.37M</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>+$2.71M</t>
+          <t>+$2.82M</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>106.73</v>
+        <v>3943.49</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>174</v>
+        <v>363</v>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>+$1.56M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>-$2.49M</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>+$2.70M</t>
+          <t>+$2.71M</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -4904,108 +4941,104 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
+        <v>106.73</v>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>174</v>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>+$1.56M</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>+$2.70M</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
         <v>107.35</v>
       </c>
-      <c r="C54" s="2" t="n">
+      <c r="C55" s="2" t="n">
         <v>175</v>
       </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E54" s="8" t="inlineStr">
+      <c r="E55" s="8" t="inlineStr">
         <is>
           <t>+$2.07M</t>
         </is>
       </c>
-      <c r="F54" s="3" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>+$2.08M</t>
         </is>
       </c>
-      <c r="G54" s="3" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B55" s="5" t="n">
+      <c r="B56" s="5" t="n">
         <v>98.15000000000001</v>
       </c>
-      <c r="C55" s="5" t="n">
+      <c r="C56" s="5" t="n">
         <v>160</v>
       </c>
-      <c r="D55" s="6" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="E56" s="7" t="inlineStr">
         <is>
           <t>-$1.27M</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>+$1.88M</t>
         </is>
       </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H55" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="n">
-        <v>100.6</v>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>164</v>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>-$1.28M</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>+$1.87M</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -5018,10 +5051,10 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>99.98999999999999</v>
+        <v>100.6</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
@@ -5030,12 +5063,12 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>-$92.13K</t>
+          <t>-$1.28M</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>+$999.85K</t>
+          <t>+$1.87M</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -5045,7 +5078,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5056,24 +5089,24 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>105.51</v>
+        <v>99.98999999999999</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>+$128.62K</t>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>-$92.13K</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>+$736.83K</t>
+          <t>+$999.85K</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -5083,83 +5116,83 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>105.51</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>172</v>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>+$128.62K</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>+$736.83K</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B59" s="2" t="n">
+      <c r="B60" s="2" t="n">
         <v>4061.6</v>
       </c>
-      <c r="C59" s="2" t="n">
+      <c r="C60" s="2" t="n">
         <v>82.5</v>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E59" s="8" t="inlineStr">
+      <c r="E60" s="8" t="inlineStr">
         <is>
           <t>+$97.36K</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>+$498.37K</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr">
+      <c r="H60" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="n">
-        <v>29044.49</v>
-      </c>
-      <c r="C60" s="5" t="n">
-        <v>29500</v>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E60" s="9" t="inlineStr">
-        <is>
-          <t>+$257.57K</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>+$459.86K</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5170,108 +5203,112 @@
         </is>
       </c>
       <c r="B61" s="5" t="n">
+        <v>29044.49</v>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>29500</v>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E61" s="9" t="inlineStr">
+        <is>
+          <t>+$257.57K</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>+$459.86K</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="n">
         <v>28944.49</v>
       </c>
-      <c r="C61" s="5" t="n">
+      <c r="C62" s="5" t="n">
         <v>29400</v>
       </c>
-      <c r="D61" s="6" t="inlineStr">
+      <c r="D62" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E61" s="9" t="inlineStr">
+      <c r="E62" s="9" t="inlineStr">
         <is>
           <t>+$295.79K</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="F62" s="6" t="inlineStr">
         <is>
           <t>+$403.99K</t>
         </is>
       </c>
-      <c r="G61" s="6" t="inlineStr">
+      <c r="G62" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H61" s="6" t="inlineStr">
+      <c r="H62" s="6" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="n">
-        <v>4110.83</v>
-      </c>
-      <c r="C62" s="2" t="n">
-        <v>83.5</v>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>+$184.53K</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>+$311.09K</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H62" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>28919.49</v>
+        <v>4110.83</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>29375</v>
+        <v>83.5</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>+$152.31K</t>
+          <t>+$184.53K</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>+$185.24K</t>
+          <t>+$311.09K</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -5280,10 +5317,10 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>28994.49</v>
+        <v>28919.49</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>29450</v>
+        <v>29375</v>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
@@ -5292,12 +5329,12 @@
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>+$96.44K</t>
+          <t>+$152.31K</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>+$178.77K</t>
+          <t>+$185.24K</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -5314,24 +5351,24 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>28844.49</v>
+        <v>28994.49</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>29300</v>
+        <v>29450</v>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>-$84.68K</t>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>+$96.44K</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>+$152.89K</t>
+          <t>+$178.77K</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -5348,24 +5385,24 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>29094.49</v>
+        <v>28844.49</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>29550</v>
+        <v>29300</v>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>+$85.86K</t>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>-$84.68K</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>+$130.55K</t>
+          <t>+$152.89K</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -5382,10 +5419,10 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>28964.49</v>
+        <v>29094.49</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>29420</v>
+        <v>29550</v>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
@@ -5394,24 +5431,20 @@
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>+$17.94K</t>
+          <t>+$85.86K</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>+$36.75K</t>
+          <t>+$130.55K</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -5420,39 +5453,77 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
+        <v>28964.49</v>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>29420</v>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>+$17.94K</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>+$36.75K</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
         <v>29084.49</v>
       </c>
-      <c r="C68" s="2" t="n">
+      <c r="C69" s="2" t="n">
         <v>29540</v>
       </c>
-      <c r="D68" s="3" t="inlineStr">
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>-$7.64K</t>
         </is>
       </c>
-      <c r="F68" s="3" t="inlineStr">
+      <c r="F69" s="3" t="inlineStr">
         <is>
           <t>+$27.64K</t>
         </is>
       </c>
-      <c r="G68" s="3" t="inlineStr">
+      <c r="G69" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H68" s="3" t="inlineStr">
+      <c r="H69" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H68"/>
+  <autoFilter ref="A1:H69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>